<commit_message>
Fix config dropdown validation scopes
</commit_message>
<xml_diff>
--- a/IBIS_Codex_READY_FOR_T2B_Package/inputs/config/ibis_config.xlsx
+++ b/IBIS_Codex_READY_FOR_T2B_Package/inputs/config/ibis_config.xlsx
@@ -3089,28 +3089,28 @@
     <mergeCell ref="A14:D14"/>
   </mergeCells>
   <dataValidations count="8">
-    <dataValidation sqref="B11:B30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="B11:B12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"DRV,RCV,BOTH"</formula1>
     </dataValidation>
-    <dataValidation sqref="B42:B55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="B42:B48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"DRV,RCV,BOTH"</formula1>
     </dataValidation>
-    <dataValidation sqref="B51:B60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="B51:B54" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"DRV,RCV,BOTH"</formula1>
     </dataValidation>
-    <dataValidation sqref="B57:B65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="B57:B59" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"DRV,RCV"</formula1>
     </dataValidation>
-    <dataValidation sqref="C57:C65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="C57:C59" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"drv_se,drv_diff,rcv_se,rcv_diff"</formula1>
     </dataValidation>
-    <dataValidation sqref="B62:B66" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="B62:B67" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"DRV,RCV,BOTH"</formula1>
     </dataValidation>
-    <dataValidation sqref="C62:C66" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="C62:C67" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"MAX,TYP,MIN,ALL"</formula1>
     </dataValidation>
-    <dataValidation sqref="C70:C73" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="C70:C74" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"POWER_DOMAIN"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>